<commit_message>
n8n board refresh 2026-08-04T17:42:42Z
</commit_message>
<xml_diff>
--- a/app/reports/ASPS_research.xlsx
+++ b/app/reports/ASPS_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-03 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-04 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>5.695</v>
+        <v>5.047</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04690000057220459</v>
+        <v>0.0463100004196167</v>
       </c>
     </row>
     <row r="6">
@@ -1197,7 +1197,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>11420206.49692713</v>
+        <v>11420206.06300773</v>
       </c>
     </row>
     <row r="36">
@@ -1218,7 +1218,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>5.695</v>
+        <v>5.047</v>
       </c>
     </row>
     <row r="38">
@@ -1497,11 +1497,11 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>65038076</v>
+        <v>57637780</v>
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31" t="n">
-        <v>22.65</v>
+        <v>22.66</v>
       </c>
       <c r="F5" s="31" t="n">
         <v>1.25</v>
@@ -1519,16 +1519,16 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>122019576</v>
+        <v>120162752</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>9.543568</v>
+        <v>9.398339999999999</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>5.573</v>
+        <v>5.286</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>1.34</v>
+        <v>1.271</v>
       </c>
     </row>
     <row r="7">
@@ -1543,14 +1543,14 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>75588176</v>
+        <v>74146432</v>
       </c>
       <c r="D7" s="33" t="n"/>
       <c r="E7" s="33" t="n">
-        <v>25.205</v>
+        <v>25.132</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>8.182</v>
+        <v>8.157999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -1565,16 +1565,16 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>149271776</v>
+        <v>151836576</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>8.712574999999999</v>
+        <v>8.654971</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>10.816</v>
+        <v>11.106</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>1.923</v>
+        <v>1.975</v>
       </c>
     </row>
     <row r="9">
@@ -1589,14 +1589,14 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>48303040</v>
+        <v>48365448</v>
       </c>
       <c r="D9" s="33" t="n"/>
       <c r="E9" s="33" t="n">
-        <v>7.787</v>
+        <v>7.811</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>2.633</v>
+        <v>2.641</v>
       </c>
     </row>
     <row r="10">
@@ -1611,12 +1611,12 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>68525056</v>
+        <v>71409824</v>
       </c>
       <c r="D10" s="33" t="n"/>
       <c r="E10" s="33" t="n"/>
       <c r="F10" s="33" t="n">
-        <v>97.16800000000001</v>
+        <v>97.215</v>
       </c>
     </row>
     <row r="11">
@@ -1631,14 +1631,14 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>14217453</v>
+        <v>13776102</v>
       </c>
       <c r="D11" s="33" t="n"/>
       <c r="E11" s="33" t="n">
-        <v>-54.02</v>
+        <v>-53.138</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>0.537</v>
+        <v>0.528</v>
       </c>
     </row>
     <row r="12">
@@ -1653,14 +1653,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>223564032</v>
+        <v>231534912</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
-        <v>-5.11</v>
+        <v>-5.655</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>196.647</v>
+        <v>217.616</v>
       </c>
     </row>
     <row r="13">
@@ -1675,14 +1675,14 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>152304592</v>
+        <v>151736288</v>
       </c>
       <c r="D13" s="33" t="n"/>
       <c r="E13" s="33" t="n">
-        <v>13.389</v>
+        <v>13.495</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>4.817</v>
+        <v>4.855</v>
       </c>
     </row>
     <row r="15">

</xml_diff>